<commit_message>
guardado, lectura de reglas y estilo de excel listo, falta funcionalidad de borrar reglas
</commit_message>
<xml_diff>
--- a/Galic2.xlsx
+++ b/Galic2.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="359">
   <si>
     <t xml:space="preserve">Resumen de Cuenta Corriente en Pesos  </t>
@@ -91,6 +91,9 @@
     <t>Saldo</t>
   </si>
   <si>
+    <t>Clasificacion</t>
+  </si>
+  <si>
     <t>02/01/23</t>
   </si>
   <si>
@@ -103,10 +106,10 @@
     <t>625.110,79</t>
   </si>
   <si>
-    <t xml:space="preserve">PAGO DE SERVICIOS VISA- 450832800184- 589244000756014567-</t>
+    <t>Proveedores</t>
+  </si>
+  <si>
+    <t>PAGO DE SERVICIOS VISA 450832800184 589244000756014567</t>
   </si>
   <si>
     <t>-66.840,54</t>
@@ -115,10 +118,10 @@
     <t>558.270,25</t>
   </si>
   <si>
-    <t xml:space="preserve">PAGO DE SERVICIOS AMEX- 377797800393- 589244000756014567-</t>
+    <t>Particular</t>
+  </si>
+  <si>
+    <t>PAGO DE SERVICIOS AMEX 377797800393 589244000756014567</t>
   </si>
   <si>
     <t>-32.366,26</t>
@@ -127,12 +130,7 @@
     <t>525.903,99</t>
   </si>
   <si>
-    <t xml:space="preserve">TRF INMED PROVEED JULIO NOE ARIAS SOCI- 30671839060- 0147388820- FACTURAS- BANCO DE GALICIA Y B-</t>
+    <t>TRF INMED PROVEED JULIO NOE ARIAS SOCI 30671839060 0147388820 FACTURAS BANCO DE GALICIA Y B</t>
   </si>
   <si>
     <t>-99.996,16</t>
@@ -141,12 +139,7 @@
     <t>425.907,83</t>
   </si>
   <si>
-    <t xml:space="preserve">TRF INMED PROVEED CML S.R.L.- 30711605513- 0147389305- VARIOS- BANCO PATAGONIA S.A.-</t>
+    <t>TRF INMED PROVEED CML S.R.L. 30711605513 0147389305 VARIOS BANCO PATAGONIA S.A.</t>
   </si>
   <si>
     <t>-9.000,00</t>
@@ -164,9 +157,10 @@
     <t>415.620,63</t>
   </si>
   <si>
-    <t xml:space="preserve">COMISION MANTENIMIENTO CTA. CTE/CCE- Diciembre 2022-</t>
+    <t>Deb. Ley 25413</t>
+  </si>
+  <si>
+    <t>COMISION MANTENIMIENTO CTA. CTE/CCE Diciembre 2022</t>
   </si>
   <si>
     <t>-5.625,00</t>
@@ -175,8 +169,10 @@
     <t>409.995,63</t>
   </si>
   <si>
-    <t xml:space="preserve">COM. MOVIMIENTOS Diciembre 2022-</t>
+    <t>Gastos Brios</t>
+  </si>
+  <si>
+    <t>COM. MOVIMIENTOS Diciembre 2022</t>
   </si>
   <si>
     <t>-330,00</t>
@@ -194,6 +190,9 @@
     <t>409.496,88</t>
   </si>
   <si>
+    <t>PERC. IVA</t>
+  </si>
+  <si>
     <t>-1.181,25</t>
   </si>
   <si>
@@ -212,9 +211,7 @@
     <t>408.221,40</t>
   </si>
   <si>
-    <t xml:space="preserve">INTERESES SOBRE SALDOS DEUDORES- Diciembre 2022-</t>
+    <t>INTERESES SOBRE SALDOS DEUDORES Diciembre 2022</t>
   </si>
   <si>
     <t>-7.887,89</t>
@@ -223,6 +220,9 @@
     <t>400.333,51</t>
   </si>
   <si>
+    <t>Intereses</t>
+  </si>
+  <si>
     <t>-118,32</t>
   </si>
   <si>
@@ -244,6 +244,9 @@
     <t>399.133,58</t>
   </si>
   <si>
+    <t>SIN CLASIFICAR</t>
+  </si>
+  <si>
     <t>-30,72</t>
   </si>
   <si>
@@ -253,11 +256,7 @@
     <t>03/01/23</t>
   </si>
   <si>
-    <t xml:space="preserve">DEB. AUTOM. DE SERV. TELECOM ARGENTIN- CONSUMOS- 000000000000368- 5787146454-</t>
+    <t>DEB. AUTOM. DE SERV. TELECOM ARGENTIN CONSUMOS 000000000000368 5787146454</t>
   </si>
   <si>
     <t>-19.254,24</t>
@@ -266,12 +265,7 @@
     <t>379.848,62</t>
   </si>
   <si>
-    <t xml:space="preserve">TRF INMED PROVEED MARCHENA GABRIEL JUL- 20119643687- 0147460723- VARIOS- BANCO SANTANDER RIO-</t>
+    <t>TRF INMED PROVEED MARCHENA GABRIEL JUL 20119643687 0147460723 VARIOS BANCO SANTANDER RIO</t>
   </si>
   <si>
     <t>-5.294,00</t>
@@ -280,12 +274,7 @@
     <t>374.554,62</t>
   </si>
   <si>
-    <t xml:space="preserve">TRF INMED PROVEED MARCHENA GABRIEL JUL- 20119643687- 0147461501- VARIOS- BANCO SANTANDER RIO-</t>
+    <t>TRF INMED PROVEED MARCHENA GABRIEL JUL 20119643687 0147461501 VARIOS BANCO SANTANDER RIO</t>
   </si>
   <si>
     <t>-9.529,00</t>
@@ -294,12 +283,7 @@
     <t>365.025,62</t>
   </si>
   <si>
-    <t xml:space="preserve">TRF INMED PROVEED MARCHENA GABRIEL JUL- 20119643687- 0147461770- VARIOS- BANCO SANTANDER RIO-</t>
+    <t>TRF INMED PROVEED MARCHENA GABRIEL JUL 20119643687 0147461770 VARIOS BANCO SANTANDER RIO</t>
   </si>
   <si>
     <t>-69.924,00</t>
@@ -317,8 +301,7 @@
     <t>04/01/23</t>
   </si>
   <si>
-    <t xml:space="preserve">RESCATE FIMA FIMA PREMIUM CLASE A-</t>
+    <t>RESCATE FIMA FIMA PREMIUM CLASE A</t>
   </si>
   <si>
     <t>1.508.988,00</t>
@@ -327,10 +310,10 @@
     <t>1.803.738,10</t>
   </si>
   <si>
-    <t xml:space="preserve">SERVICIO ACREDITAMIENTO DE HABERES- 0147604122- ACRED.HABERES-</t>
+    <t>Rescate fondos FIMA</t>
+  </si>
+  <si>
+    <t>SERVICIO ACREDITAMIENTO DE HABERES 0147604122 ACRED.HABERES</t>
   </si>
   <si>
     <t>-1.799.737,80</t>
@@ -339,13 +322,13 @@
     <t>4.000,30</t>
   </si>
   <si>
+    <t>HABERES</t>
+  </si>
+  <si>
     <t>09/01/23</t>
   </si>
   <si>
-    <t xml:space="preserve">SNP PAGO A PROVEEDORES GBO.DE LA PROVIN- 30671853535- BANCO RIOJA SOCIEDAD-</t>
+    <t>SNP PAGO A PROVEEDORES GBO.DE LA PROVIN 30671853535 BANCO RIOJA SOCIEDAD</t>
   </si>
   <si>
     <t>340.843,40</t>
@@ -354,6 +337,9 @@
     <t>338.760,59</t>
   </si>
   <si>
+    <t>Transferencias</t>
+  </si>
+  <si>
     <t>IMP. CRE. LEY 25413 REDUC.</t>
   </si>
   <si>
@@ -363,8 +349,10 @@
     <t>337.608,54</t>
   </si>
   <si>
-    <t xml:space="preserve">PAGO VISA EMPRESA D.A. AL VTO BUSINESS-</t>
+    <t>Cred Ley 25413</t>
+  </si>
+  <si>
+    <t>PAGO VISA EMPRESA D.A. AL VTO BUSINESS</t>
   </si>
   <si>
     <t>-270.707,84</t>
@@ -373,6 +361,9 @@
     <t>66.900,70</t>
   </si>
   <si>
+    <t>Tarj VISA</t>
+  </si>
+  <si>
     <t>-914,99</t>
   </si>
   <si>
@@ -382,12 +373,7 @@
     <t>10/01/23</t>
   </si>
   <si>
-    <t xml:space="preserve">TRANSF. A TERCEROS DIRECCION GRAL DE IN- 30711022909- 0148088499- VARIOS- BANCO RIOJA SOCIEDAD-</t>
+    <t>TRANSF. A TERCEROS DIRECCION GRAL DE IN 30711022909 0148088499 VARIOS BANCO RIOJA SOCIEDAD</t>
   </si>
   <si>
     <t>-100,00</t>
@@ -396,12 +382,7 @@
     <t>65.885,71</t>
   </si>
   <si>
-    <t xml:space="preserve">TRANSFERENCIA A TERCEROS ANDRES SEBASTIAN MEN- 20327618858- 0148115136- VARIOS- BANCO DE GALICIA Y B-</t>
+    <t>TRANSFERENCIA A TERCEROS ANDRES SEBASTIAN MEN 20327618858 0148115136 VARIOS BANCO DE GALICIA Y B</t>
   </si>
   <si>
     <t>-5.200,00</t>
@@ -416,11 +397,7 @@
     <t>360.685,71</t>
   </si>
   <si>
-    <t xml:space="preserve">TRANSFERENCIAS CASH PROVEEDORES- O.S.D.E.- 30546741253- BANCO DE LA NACION A-</t>
+    <t>TRANSFERENCIAS CASH PROVEEDORES O.S.D.E. 30546741253 BANCO DE LA NACION A</t>
   </si>
   <si>
     <t>1.989,00</t>
@@ -429,12 +406,7 @@
     <t>362.674,71</t>
   </si>
   <si>
-    <t xml:space="preserve">TRF INMED PROVEED MANRIQUE MARIELA NOE- 27294491169- 0148149053- VARIOS- BANCO HIPOTECARIO S.-</t>
+    <t>TRF INMED PROVEED MANRIQUE MARIELA NOE 27294491169 0148149053 VARIOS BANCO HIPOTECARIO S.</t>
   </si>
   <si>
     <t>-111.300,00</t>
@@ -443,12 +415,7 @@
     <t>251.374,71</t>
   </si>
   <si>
-    <t xml:space="preserve">TRANSF. A TERCEROS MARIACA   NATALIA FA- 27282430792- 0148149729- VARIOS- BANCO BBVA ARGENTINA-</t>
+    <t>TRANSF. A TERCEROS MARIACA   NATALIA FA 27282430792 0148149729 VARIOS BANCO BBVA ARGENTINA</t>
   </si>
   <si>
     <t>-12.800,00</t>
@@ -457,12 +424,7 @@
     <t>238.574,71</t>
   </si>
   <si>
-    <t xml:space="preserve">TRANSF. A TERCEROS SIMONETTI IGNACIO NI- 20431505534- 0148151291- VARIOS- BANCO DE LA NACION A-</t>
+    <t>TRANSF. A TERCEROS SIMONETTI IGNACIO NI 20431505534 0148151291 VARIOS BANCO DE LA NACION A</t>
   </si>
   <si>
     <t>-41.300,00</t>
@@ -471,12 +433,7 @@
     <t>197.274,71</t>
   </si>
   <si>
-    <t xml:space="preserve">TRANSF. A TERCEROS VILLEGAS CASTRO ALDO- 20308358616- 0148153224- VARIOS- BANCO RIOJA SOCIEDAD-</t>
+    <t>TRANSF. A TERCEROS VILLEGAS CASTRO ALDO 20308358616 0148153224 VARIOS BANCO RIOJA SOCIEDAD</t>
   </si>
   <si>
     <t>-59.550,00</t>
@@ -485,12 +442,7 @@
     <t>137.724,71</t>
   </si>
   <si>
-    <t xml:space="preserve">TRANSF. A TERCEROS MATUS MARIA ELISA- 27296940947- 0148153760- VARIOS- BANCO DE LA NACION A-</t>
+    <t>TRANSF. A TERCEROS MATUS MARIA ELISA 27296940947 0148153760 VARIOS BANCO DE LA NACION A</t>
   </si>
   <si>
     <t>-35.000,00</t>
@@ -499,12 +451,7 @@
     <t>102.724,71</t>
   </si>
   <si>
-    <t xml:space="preserve">TRANSF. A TERCEROS CABRERA DIAZ SILVIA- 27311288380- 0148155146- VARIOS- BANCO RIOJA SOCIEDAD-</t>
+    <t>TRANSF. A TERCEROS CABRERA DIAZ SILVIA 27311288380 0148155146 VARIOS BANCO RIOJA SOCIEDAD</t>
   </si>
   <si>
     <t>-87.360,00</t>
@@ -528,11 +475,7 @@
     <t>12/01/23</t>
   </si>
   <si>
-    <t xml:space="preserve">TRANSFERENCIA DE TERCEROS BRAVO JORGE LUIS- 23119714559- PRESTAMOS- OPERACION 2410816525-</t>
+    <t>TRANSFERENCIA DE TERCEROS BRAVO JORGE LUIS 23119714559 PRESTAMOS OPERACION 2410816525</t>
   </si>
   <si>
     <t>161.000,00</t>
@@ -541,12 +484,7 @@
     <t>174.152,17</t>
   </si>
   <si>
-    <t xml:space="preserve">TRF INMED PROVEED GAMBOA GARCIA ABEL G- 23190200779- 0148334028- VARIOS- BANCO SANTANDER RIO-</t>
+    <t>TRF INMED PROVEED GAMBOA GARCIA ABEL G 23190200779 0148334028 VARIOS BANCO SANTANDER RIO</t>
   </si>
   <si>
     <t>-160.800,00</t>
@@ -555,12 +493,7 @@
     <t>13.352,17</t>
   </si>
   <si>
-    <t xml:space="preserve">TRF INMED PROVEED QUIMICA RIOJA SRL- 30715631837- 0148334855- VARIOS- BANCO SANTANDER RIO-</t>
+    <t>TRF INMED PROVEED QUIMICA RIOJA SRL 30715631837 0148334855 VARIOS BANCO SANTANDER RIO</t>
   </si>
   <si>
     <t>-10.859,76</t>
@@ -584,11 +517,7 @@
     <t>13/01/23</t>
   </si>
   <si>
-    <t xml:space="preserve">TRANSFERENCIA DE TERCEROS JORGE LUIS BRAVO- 23119714559- PRESTAMOS- BANCO DE GALICIA Y B-</t>
+    <t>TRANSFERENCIA DE TERCEROS JORGE LUIS BRAVO 23119714559 PRESTAMOS BANCO DE GALICIA Y B</t>
   </si>
   <si>
     <t>39.300,00</t>
@@ -597,12 +526,7 @@
     <t>40.668,02</t>
   </si>
   <si>
-    <t xml:space="preserve">TRANSF. A TERCEROS MANRIQUE MARIELA NOE- 27294491169- 0148527507- HONORARIOS- BANCO HIPOTECARIO S.-</t>
+    <t>TRANSF. A TERCEROS MANRIQUE MARIELA NOE 27294491169 0148527507 HONORARIOS BANCO HIPOTECARIO S.</t>
   </si>
   <si>
     <t>-39.200,00</t>
@@ -626,11 +550,7 @@
     <t>17/01/23</t>
   </si>
   <si>
-    <t xml:space="preserve">TRANSFERENCIAS CASH PROVEEDORES- Conf.de Asoc. de Dia- 30694436591- HSBC BANK ARGENTINA-</t>
+    <t>TRANSFERENCIAS CASH PROVEEDORES Conf.de Asoc. de Dia 30694436591 HSBC BANK ARGENTINA</t>
   </si>
   <si>
     <t>191.654,23</t>
@@ -648,12 +568,7 @@
     <t>18/01/23</t>
   </si>
   <si>
-    <t xml:space="preserve">TRANSFERENCIA A TERCEROS HORACIO ESTEBAN BUSL- 20249397882- 0148837098- VARIOS- BANCO DE GALICIA Y B-</t>
+    <t>TRANSFERENCIA A TERCEROS HORACIO ESTEBAN BUSL 20249397882 0148837098 VARIOS BANCO DE GALICIA Y B</t>
   </si>
   <si>
     <t>-16.300,00</t>
@@ -662,12 +577,7 @@
     <t>175.909,13</t>
   </si>
   <si>
-    <t xml:space="preserve">TRF INMED PROVEED GUEMES LUIS ALEJANDR- 20331730956- 0148840189- VARIOS- BANCO SANTANDER RIO-</t>
+    <t>TRF INMED PROVEED GUEMES LUIS ALEJANDR 20331730956 0148840189 VARIOS BANCO SANTANDER RIO</t>
   </si>
   <si>
     <t>-10.500,00</t>
@@ -676,12 +586,7 @@
     <t>165.409,13</t>
   </si>
   <si>
-    <t xml:space="preserve">TRANSFERENCIA A TERCEROS JORGE LUIS BRAVO- 23119714559- 0148843662- VARIOS- BANCO DE GALICIA Y B-</t>
+    <t>TRANSFERENCIA A TERCEROS JORGE LUIS BRAVO 23119714559 0148843662 VARIOS BANCO DE GALICIA Y B</t>
   </si>
   <si>
     <t>-30.000,00</t>
@@ -699,8 +604,7 @@
     <t>19/01/23</t>
   </si>
   <si>
-    <t xml:space="preserve">ANUL. PAGO COMERCIOS VISA EST.:0046459087-</t>
+    <t>ANUL. PAGO COMERCIOS VISA EST.:0046459087</t>
   </si>
   <si>
     <t>-4.338,76</t>
@@ -709,12 +613,7 @@
     <t>130.878,39</t>
   </si>
   <si>
-    <t xml:space="preserve">TRF INMED PROVEED MARCHENA GABRIEL JUL- 20119643687- 0148888676- VARIOS- BANCO SANTANDER RIO-</t>
+    <t>TRF INMED PROVEED MARCHENA GABRIEL JUL 20119643687 0148888676 VARIOS BANCO SANTANDER RIO</t>
   </si>
   <si>
     <t>125.584,39</t>
@@ -726,8 +625,7 @@
     <t>125.566,50</t>
   </si>
   <si>
-    <t xml:space="preserve">DEV.IMP.CRE.LEY 25413-ALIC.REDUCIDA-</t>
+    <t>DEV.IMP.CRE.LEY 25413-ALIC.REDUCIDA</t>
   </si>
   <si>
     <t>14,67</t>
@@ -739,8 +637,7 @@
     <t>20/01/23</t>
   </si>
   <si>
-    <t xml:space="preserve">EXTRACCION CAJERO 4173090000632848-</t>
+    <t>EXTRACCION CAJERO 4173090000632848</t>
   </si>
   <si>
     <t>0271</t>
@@ -752,12 +649,10 @@
     <t>112.381,17</t>
   </si>
   <si>
-    <t xml:space="preserve">PAGO PEI RAPIPAGO- 30643990632- LINK- 4173090000632848- PAGO CON TRANSF.-</t>
+    <t>Extracción</t>
+  </si>
+  <si>
+    <t>PAGO PEI RAPIPAGO 30643990632 LINK 4173090000632848 PAGO CON TRANSF.</t>
   </si>
   <si>
     <t>0002</t>
@@ -769,8 +664,7 @@
     <t>95.145,17</t>
   </si>
   <si>
-    <t xml:space="preserve">IMPUESTO DEB.LEY 25413 EXTRAC. EFEC-</t>
+    <t>IMPUESTO DEB.LEY 25413 EXTRAC. EFEC</t>
   </si>
   <si>
     <t>-44,62</t>
@@ -791,8 +685,7 @@
     <t>29.994,77</t>
   </si>
   <si>
-    <t xml:space="preserve">COMISION EXTRACCION EN EFECTIVO-</t>
+    <t>COMISION EXTRACCION EN EFECTIVO</t>
   </si>
   <si>
     <t>-264,00</t>
@@ -816,12 +709,7 @@
     <t>24/01/23</t>
   </si>
   <si>
-    <t xml:space="preserve">TRF INMED PROVEED SUPERCANAL S A- 30611182526- 0149216932- VARIOS- BANCO RIOJA SOCIEDAD-</t>
+    <t>TRF INMED PROVEED SUPERCANAL S A 30611182526 0149216932 VARIOS BANCO RIOJA SOCIEDAD</t>
   </si>
   <si>
     <t>-12.318,00</t>
@@ -830,9 +718,7 @@
     <t>17.136,19</t>
   </si>
   <si>
-    <t xml:space="preserve">TRANSF. AFIP 0149248608- VEP 1049430514-</t>
+    <t>TRANSF. AFIP 0149248608 VEP 1049430514</t>
   </si>
   <si>
     <t>-14.307,08</t>
@@ -841,6 +727,9 @@
     <t>2.829,11</t>
   </si>
   <si>
+    <t>ARCA</t>
+  </si>
+  <si>
     <t>206.786,49</t>
   </si>
   <si>
@@ -862,12 +751,7 @@
     <t>25/01/23</t>
   </si>
   <si>
-    <t xml:space="preserve">TRF INMED PROVEED QUIMICA RIOJA SRL- 30715631837- 0149343969- VARIOS- BANCO SANTANDER RIO-</t>
+    <t>TRF INMED PROVEED QUIMICA RIOJA SRL 30715631837 0149343969 VARIOS BANCO SANTANDER RIO</t>
   </si>
   <si>
     <t>-5.000,00</t>
@@ -894,11 +778,7 @@
     <t>140.359,77</t>
   </si>
   <si>
-    <t xml:space="preserve">DEB. AUTOM. DE SERV. AFIP- PLANRG5101- R5101Q118078009- 33714315299-</t>
+    <t>DEB. AUTOM. DE SERV. AFIP PLANRG5101 R5101Q118078009 33714315299</t>
   </si>
   <si>
     <t>-14.298,42</t>
@@ -907,11 +787,7 @@
     <t>126.061,35</t>
   </si>
   <si>
-    <t xml:space="preserve">DEB. AUTOM. DE SERV. AFIP- PLANRG4816- R4816O155835026- 33714315299-</t>
+    <t>DEB. AUTOM. DE SERV. AFIP PLANRG4816 R4816O155835026 33714315299</t>
   </si>
   <si>
     <t>-22.393,18</t>
@@ -920,11 +796,7 @@
     <t>103.668,17</t>
   </si>
   <si>
-    <t xml:space="preserve">DEB. AUTOM. DE SERV. AFIP- PLANRG4816- R4816O151277026- 33714315299-</t>
+    <t>DEB. AUTOM. DE SERV. AFIP PLANRG4816 R4816O151277026 33714315299</t>
   </si>
   <si>
     <t>-100.469,05</t>
@@ -933,11 +805,7 @@
     <t>3.199,12</t>
   </si>
   <si>
-    <t xml:space="preserve">TRANSFERENCIAS CASH PROVEEDORES- Conf.de Asoc.de Dial- 30694436591- BANCO DE LA NACION A-</t>
+    <t>TRANSFERENCIAS CASH PROVEEDORES Conf.de Asoc.de Dial 30694436591 BANCO DE LA NACION A</t>
   </si>
   <si>
     <t>1.311.119,15</t>
@@ -976,10 +844,7 @@
     <t>2.261.244,27</t>
   </si>
   <si>
-    <t xml:space="preserve">SERVICIO ACREDITAMIENTO DE HABERES- 0149478186- ACRED.HABERES-</t>
+    <t>SERVICIO ACREDITAMIENTO DE HABERES 0149478186 ACRED.HABERES</t>
   </si>
   <si>
     <t>-771.316,20</t>
@@ -988,12 +853,7 @@
     <t>1.489.928,07</t>
   </si>
   <si>
-    <t xml:space="preserve">TRF INMED PROVEED NIETO RUIZ HUGO ADRI- 20202532528- 0149483807- VARIOS- BANCO SANTANDER RIO-</t>
+    <t>TRF INMED PROVEED NIETO RUIZ HUGO ADRI 20202532528 0149483807 VARIOS BANCO SANTANDER RIO</t>
   </si>
   <si>
     <t>-90.000,00</t>
@@ -1002,12 +862,7 @@
     <t>1.399.928,07</t>
   </si>
   <si>
-    <t xml:space="preserve">TRF INMED PROVEED GAMBOA GARCIA ABEL G- 23190200779- 0149487743- VARIOS- BANCO SANTANDER RIO-</t>
+    <t>TRF INMED PROVEED GAMBOA GARCIA ABEL G 23190200779 0149487743 VARIOS BANCO SANTANDER RIO</t>
   </si>
   <si>
     <t>-157.720,00</t>
@@ -1031,12 +886,7 @@
     <t>1.204.208,07</t>
   </si>
   <si>
-    <t xml:space="preserve">TRF INMED PROVEED JORGE LUIS BRAVO- 23119714559- 0149510658- VARIOS- BANCO DE GALICIA Y B-</t>
+    <t>TRF INMED PROVEED JORGE LUIS BRAVO 23119714559 0149510658 VARIOS BANCO DE GALICIA Y B</t>
   </si>
   <si>
     <t>-70.300,00</t>
@@ -1045,9 +895,7 @@
     <t>1.133.908,07</t>
   </si>
   <si>
-    <t xml:space="preserve">TRANSF. AFIP 0149511622- VEP 1050857745-</t>
+    <t>TRANSF. AFIP 0149511622 VEP 1050857745</t>
   </si>
   <si>
     <t>-297.067,81</t>
@@ -1056,10 +904,7 @@
     <t>836.840,26</t>
   </si>
   <si>
-    <t xml:space="preserve">SERVICIO ACREDITAMIENTO DE HABERES- 0149534692- SUELDO ANUAL COMPLEM-</t>
+    <t>SERVICIO ACREDITAMIENTO DE HABERES 0149534692 SUELDO ANUAL COMPLEM</t>
   </si>
   <si>
     <t>-602.496,50</t>
@@ -1068,12 +913,7 @@
     <t>234.343,76</t>
   </si>
   <si>
-    <t xml:space="preserve">TRF INMED PROVEED BARRIA NIEVAS SEBAST- 20387614762- 0149535305- VARIOS- BANCO SANTANDER RIO-</t>
+    <t>TRF INMED PROVEED BARRIA NIEVAS SEBAST 20387614762 0149535305 VARIOS BANCO SANTANDER RIO</t>
   </si>
   <si>
     <t>-50.000,00</t>
@@ -1118,9 +958,7 @@
     <t>700.466,33</t>
   </si>
   <si>
-    <t xml:space="preserve">ACREDITACI?N VENCIMIENTO PLAZO FIJO- 809210719798-</t>
+    <t>ACREDITACI?N VENCIMIENTO PLAZO FIJO 809210719798</t>
   </si>
   <si>
     <t>158.482,85</t>
@@ -1141,8 +979,7 @@
     <t>858.029,58</t>
   </si>
   <si>
-    <t xml:space="preserve">SUSCRIPCION FIMA FIMA PREMIUM CLASE A-</t>
+    <t>SUSCRIPCION FIMA FIMA PREMIUM CLASE A</t>
   </si>
   <si>
     <t>-160.000,00</t>
@@ -1151,12 +988,10 @@
     <t>698.029,58</t>
   </si>
   <si>
-    <t xml:space="preserve">TRF INMED PROVEED BENITEZ SEBASTIAN- 23230964149- 0149626691- FACTURAS- BANCO HIPOTECARIO S.-</t>
+    <t>Suscrip. Fondos FIMA</t>
+  </si>
+  <si>
+    <t>TRF INMED PROVEED BENITEZ SEBASTIAN 23230964149 0149626691 FACTURAS BANCO HIPOTECARIO S.</t>
   </si>
   <si>
     <t>-42.980,65</t>
@@ -1195,12 +1030,7 @@
     <t>1.059.405,35</t>
   </si>
   <si>
-    <t xml:space="preserve">TRF INMED PROVEED JULIO NOE ARIAS SOCI- 30671839060- 0149740224- FACTURAS- BANCO DE GALICIA Y B-</t>
+    <t>TRF INMED PROVEED JULIO NOE ARIAS SOCI 30671839060 0149740224 FACTURAS BANCO DE GALICIA Y B</t>
   </si>
   <si>
     <t>-11.123,52</t>
@@ -1209,12 +1039,7 @@
     <t>1.048.281,83</t>
   </si>
   <si>
-    <t xml:space="preserve">TRF INMED PROVEED QUINTEROS DOMINGO NI- 20177736555- 0149740479- FACTURAS- BANCO SANTANDER RIO-</t>
+    <t>TRF INMED PROVEED QUINTEROS DOMINGO NI 20177736555 0149740479 FACTURAS BANCO SANTANDER RIO</t>
   </si>
   <si>
     <t>-45.000,00</t>
@@ -1223,12 +1048,7 @@
     <t>1.003.281,83</t>
   </si>
   <si>
-    <t xml:space="preserve">TRF INMED PROVEED CML S.R.L.- 30711605513- 0149740829- FACTURAS- BANCO PATAGONIA S.A.-</t>
+    <t>TRF INMED PROVEED CML S.R.L. 30711605513 0149740829 FACTURAS BANCO PATAGONIA S.A.</t>
   </si>
   <si>
     <t>-5.500,01</t>
@@ -1249,10 +1069,7 @@
     <t>281.132,32</t>
   </si>
   <si>
-    <t xml:space="preserve">PAGO DE SERVICIOS VISA- 454640800377- 589244000756014567-</t>
+    <t>PAGO DE SERVICIOS VISA 454640800377 589244000756014567</t>
   </si>
   <si>
     <t>-189.702,00</t>
@@ -1284,13 +1101,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1313,15 +1135,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
   </cellXfs>
 </styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F127"/>
+  <dimension ref="A1:G127"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1417,1639 +1240,1990 @@
       <c r="F11" t="s" s="0">
         <v>23</v>
       </c>
+      <c r="G11" t="s" s="0">
+        <v>24</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E12" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F12" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="G12" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F13" t="s" s="0">
-        <v>30</v>
+        <v>32</v>
+      </c>
+      <c r="G13" t="s" s="0">
+        <v>33</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F14" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="G14" t="s" s="0">
         <v>33</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E15" t="s" s="0">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F15" t="s" s="0">
-        <v>36</v>
+        <v>39</v>
+      </c>
+      <c r="G15" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E16" t="s" s="0">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F16" t="s" s="0">
-        <v>39</v>
+        <v>42</v>
+      </c>
+      <c r="G16" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E17" t="s" s="0">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F17" t="s" s="0">
-        <v>42</v>
+        <v>45</v>
+      </c>
+      <c r="G17" t="s" s="0">
+        <v>46</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E18" t="s" s="0">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="F18" t="s" s="0">
-        <v>45</v>
+        <v>49</v>
+      </c>
+      <c r="G18" t="s" s="0">
+        <v>50</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="E19" t="s" s="0">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="F19" t="s" s="0">
-        <v>48</v>
+        <v>53</v>
+      </c>
+      <c r="G19" t="s" s="0">
+        <v>50</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="E20" t="s" s="0">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F20" t="s" s="0">
-        <v>51</v>
+        <v>56</v>
+      </c>
+      <c r="G20" t="s" s="0">
+        <v>57</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B21" t="s" s="0">
         <v>4</v>
       </c>
       <c r="E21" t="s" s="0">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="F21" t="s" s="0">
-        <v>53</v>
+        <v>59</v>
+      </c>
+      <c r="G21" t="s" s="0">
+        <v>4</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B22" t="s" s="0">
         <v>4</v>
       </c>
       <c r="E22" t="s" s="0">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="F22" t="s" s="0">
-        <v>55</v>
+        <v>61</v>
+      </c>
+      <c r="G22" t="s" s="0">
+        <v>4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E23" t="s" s="0">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="F23" t="s" s="0">
-        <v>57</v>
+        <v>63</v>
+      </c>
+      <c r="G23" t="s" s="0">
+        <v>46</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="E24" t="s" s="0">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="F24" t="s" s="0">
-        <v>60</v>
+        <v>66</v>
+      </c>
+      <c r="G24" t="s" s="0">
+        <v>67</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="E25" t="s" s="0">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="F25" t="s" s="0">
-        <v>62</v>
+        <v>69</v>
+      </c>
+      <c r="G25" t="s" s="0">
+        <v>57</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B26" t="s" s="0">
         <v>4</v>
       </c>
       <c r="E26" t="s" s="0">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="F26" t="s" s="0">
-        <v>64</v>
+        <v>71</v>
+      </c>
+      <c r="G26" t="s" s="0">
+        <v>4</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="E27" t="s" s="0">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="F27" t="s" s="0">
-        <v>67</v>
+        <v>74</v>
+      </c>
+      <c r="G27" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E28" t="s" s="0">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="F28" t="s" s="0">
-        <v>69</v>
+        <v>77</v>
+      </c>
+      <c r="G28" t="s" s="0">
+        <v>46</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="E29" t="s" s="0">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="F29" t="s" s="0">
-        <v>73</v>
+        <v>81</v>
+      </c>
+      <c r="G29" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="E30" t="s" s="0">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F30" t="s" s="0">
-        <v>76</v>
+        <v>84</v>
+      </c>
+      <c r="G30" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="E31" t="s" s="0">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="F31" t="s" s="0">
-        <v>79</v>
+        <v>87</v>
+      </c>
+      <c r="G31" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="E32" t="s" s="0">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="F32" t="s" s="0">
-        <v>82</v>
+        <v>90</v>
+      </c>
+      <c r="G32" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E33" t="s" s="0">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="F33" t="s" s="0">
-        <v>84</v>
+        <v>92</v>
+      </c>
+      <c r="G33" t="s" s="0">
+        <v>46</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="D34" t="s" s="0">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="F34" t="s" s="0">
-        <v>88</v>
+        <v>96</v>
+      </c>
+      <c r="G34" t="s" s="0">
+        <v>97</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="E35" t="s" s="0">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="F35" t="s" s="0">
-        <v>91</v>
+        <v>100</v>
+      </c>
+      <c r="G35" t="s" s="0">
+        <v>101</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="B36" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F36" s="0"/>
+      <c r="G36" t="s" s="0">
+        <v>46</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="D37" t="s" s="0">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="F37" t="s" s="0">
-        <v>95</v>
+        <v>105</v>
+      </c>
+      <c r="G37" t="s" s="0">
+        <v>106</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="B38" t="s" s="0">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="E38" t="s" s="0">
-        <v>97</v>
+        <v>108</v>
       </c>
       <c r="F38" t="s" s="0">
-        <v>98</v>
+        <v>109</v>
+      </c>
+      <c r="G38" t="s" s="0">
+        <v>110</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="B39" t="s" s="0">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="E39" t="s" s="0">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="F39" t="s" s="0">
-        <v>101</v>
+        <v>113</v>
+      </c>
+      <c r="G39" t="s" s="0">
+        <v>114</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E40" t="s" s="0">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="F40" t="s" s="0">
-        <v>103</v>
+        <v>116</v>
+      </c>
+      <c r="G40" t="s" s="0">
+        <v>46</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="B41" t="s" s="0">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="E41" t="s" s="0">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="F41" t="s" s="0">
-        <v>107</v>
+        <v>120</v>
+      </c>
+      <c r="G41" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="E42" t="s" s="0">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="F42" t="s" s="0">
-        <v>110</v>
+        <v>123</v>
+      </c>
+      <c r="G42" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="D43" t="s" s="0">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="F43" t="s" s="0">
-        <v>112</v>
+        <v>125</v>
+      </c>
+      <c r="G43" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="0">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="D44" t="s" s="0">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="F44" t="s" s="0">
-        <v>115</v>
+        <v>128</v>
+      </c>
+      <c r="G44" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="0">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="B45" t="s" s="0">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="E45" t="s" s="0">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="F45" t="s" s="0">
-        <v>118</v>
+        <v>131</v>
+      </c>
+      <c r="G45" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="B46" t="s" s="0">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="E46" t="s" s="0">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="F46" t="s" s="0">
-        <v>121</v>
+        <v>134</v>
+      </c>
+      <c r="G46" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="B47" t="s" s="0">
-        <v>122</v>
+        <v>135</v>
       </c>
       <c r="E47" t="s" s="0">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F47" t="s" s="0">
-        <v>124</v>
+        <v>137</v>
+      </c>
+      <c r="G47" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="B48" t="s" s="0">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="E48" t="s" s="0">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="F48" t="s" s="0">
-        <v>127</v>
+        <v>140</v>
+      </c>
+      <c r="G48" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="E49" t="s" s="0">
-        <v>129</v>
+        <v>142</v>
       </c>
       <c r="F49" t="s" s="0">
-        <v>130</v>
+        <v>143</v>
+      </c>
+      <c r="G49" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="B50" t="s" s="0">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="E50" t="s" s="0">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="F50" t="s" s="0">
-        <v>133</v>
+        <v>146</v>
+      </c>
+      <c r="G50" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="0">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E51" t="s" s="0">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="F51" t="s" s="0">
-        <v>135</v>
+        <v>148</v>
+      </c>
+      <c r="G51" t="s" s="0">
+        <v>46</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="0">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="B52" t="s" s="0">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="E52" t="s" s="0">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="F52" t="s" s="0">
-        <v>137</v>
+        <v>150</v>
+      </c>
+      <c r="G52" t="s" s="0">
+        <v>110</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s" s="0">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="B53" t="s" s="0">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="D53" t="s" s="0">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="F53" t="s" s="0">
-        <v>141</v>
+        <v>154</v>
+      </c>
+      <c r="G53" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s" s="0">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="B54" t="s" s="0">
-        <v>142</v>
+        <v>155</v>
       </c>
       <c r="E54" t="s" s="0">
-        <v>143</v>
+        <v>156</v>
       </c>
       <c r="F54" t="s" s="0">
-        <v>144</v>
+        <v>157</v>
+      </c>
+      <c r="G54" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="0">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="B55" t="s" s="0">
-        <v>145</v>
+        <v>158</v>
       </c>
       <c r="E55" t="s" s="0">
-        <v>146</v>
+        <v>159</v>
       </c>
       <c r="F55" t="s" s="0">
-        <v>147</v>
+        <v>160</v>
+      </c>
+      <c r="G55" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s" s="0">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="B56" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E56" t="s" s="0">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="F56" t="s" s="0">
-        <v>149</v>
+        <v>162</v>
+      </c>
+      <c r="G56" t="s" s="0">
+        <v>46</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s" s="0">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="B57" t="s" s="0">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="E57" t="s" s="0">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="F57" t="s" s="0">
-        <v>151</v>
+        <v>164</v>
+      </c>
+      <c r="G57" t="s" s="0">
+        <v>110</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="0">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="B58" t="s" s="0">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="D58" t="s" s="0">
-        <v>154</v>
+        <v>167</v>
       </c>
       <c r="F58" t="s" s="0">
-        <v>155</v>
+        <v>168</v>
+      </c>
+      <c r="G58" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s" s="0">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="B59" t="s" s="0">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="E59" t="s" s="0">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="F59" t="s" s="0">
-        <v>158</v>
+        <v>171</v>
+      </c>
+      <c r="G59" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s" s="0">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="B60" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E60" t="s" s="0">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="F60" t="s" s="0">
-        <v>160</v>
+        <v>173</v>
+      </c>
+      <c r="G60" t="s" s="0">
+        <v>46</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s" s="0">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="B61" t="s" s="0">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="E61" t="s" s="0">
-        <v>161</v>
+        <v>174</v>
       </c>
       <c r="F61" t="s" s="0">
-        <v>162</v>
+        <v>175</v>
+      </c>
+      <c r="G61" t="s" s="0">
+        <v>110</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s" s="0">
-        <v>163</v>
+        <v>176</v>
       </c>
       <c r="B62" t="s" s="0">
-        <v>164</v>
+        <v>177</v>
       </c>
       <c r="D62" t="s" s="0">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="F62" t="s" s="0">
-        <v>166</v>
+        <v>179</v>
+      </c>
+      <c r="G62" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s" s="0">
-        <v>163</v>
+        <v>176</v>
       </c>
       <c r="B63" t="s" s="0">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="E63" t="s" s="0">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="F63" t="s" s="0">
-        <v>168</v>
+        <v>181</v>
+      </c>
+      <c r="G63" t="s" s="0">
+        <v>110</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s" s="0">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="B64" t="s" s="0">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="E64" t="s" s="0">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="F64" t="s" s="0">
-        <v>172</v>
+        <v>185</v>
+      </c>
+      <c r="G64" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s" s="0">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="B65" t="s" s="0">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="E65" t="s" s="0">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="F65" t="s" s="0">
-        <v>175</v>
+        <v>188</v>
+      </c>
+      <c r="G65" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s" s="0">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="B66" t="s" s="0">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="E66" t="s" s="0">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="F66" t="s" s="0">
-        <v>178</v>
+        <v>191</v>
+      </c>
+      <c r="G66" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s" s="0">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="B67" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E67" t="s" s="0">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="F67" t="s" s="0">
-        <v>180</v>
+        <v>193</v>
+      </c>
+      <c r="G67" t="s" s="0">
+        <v>46</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="s" s="0">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="B68" t="s" s="0">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="E68" t="s" s="0">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="F68" t="s" s="0">
-        <v>184</v>
+        <v>197</v>
+      </c>
+      <c r="G68" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="s" s="0">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="B69" t="s" s="0">
-        <v>185</v>
+        <v>198</v>
       </c>
       <c r="E69" t="s" s="0">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F69" t="s" s="0">
-        <v>186</v>
+        <v>199</v>
+      </c>
+      <c r="G69" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s" s="0">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="B70" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E70" t="s" s="0">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="F70" t="s" s="0">
-        <v>188</v>
+        <v>201</v>
+      </c>
+      <c r="G70" t="s" s="0">
+        <v>46</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s" s="0">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="B71" t="s" s="0">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="D71" t="s" s="0">
-        <v>190</v>
+        <v>203</v>
       </c>
       <c r="F71" t="s" s="0">
-        <v>191</v>
+        <v>204</v>
+      </c>
+      <c r="G71" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="s" s="0">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="B72" t="s" s="0">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="C72" t="s" s="0">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="E72" t="s" s="0">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="F72" t="s" s="0">
-        <v>196</v>
+        <v>209</v>
+      </c>
+      <c r="G72" t="s" s="0">
+        <v>210</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="s" s="0">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="B73" t="s" s="0">
-        <v>197</v>
+        <v>211</v>
       </c>
       <c r="C73" t="s" s="0">
-        <v>198</v>
+        <v>212</v>
       </c>
       <c r="E73" t="s" s="0">
-        <v>199</v>
+        <v>213</v>
       </c>
       <c r="F73" t="s" s="0">
-        <v>200</v>
+        <v>214</v>
+      </c>
+      <c r="G73" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s" s="0">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="B74" t="s" s="0">
-        <v>201</v>
+        <v>215</v>
       </c>
       <c r="E74" t="s" s="0">
-        <v>202</v>
+        <v>216</v>
       </c>
       <c r="F74" t="s" s="0">
-        <v>203</v>
+        <v>217</v>
+      </c>
+      <c r="G74" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="s" s="0">
-        <v>204</v>
+        <v>218</v>
       </c>
       <c r="B75" t="s" s="0">
-        <v>205</v>
+        <v>219</v>
       </c>
       <c r="E75" t="s" s="0">
-        <v>206</v>
+        <v>220</v>
       </c>
       <c r="F75" t="s" s="0">
-        <v>207</v>
+        <v>221</v>
+      </c>
+      <c r="G75" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s" s="0">
-        <v>204</v>
+        <v>218</v>
       </c>
       <c r="B76" t="s" s="0">
-        <v>208</v>
+        <v>222</v>
       </c>
       <c r="E76" t="s" s="0">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="F76" t="s" s="0">
-        <v>210</v>
+        <v>224</v>
+      </c>
+      <c r="G76" t="s" s="0">
+        <v>50</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="s" s="0">
-        <v>204</v>
+        <v>218</v>
       </c>
       <c r="B77" t="s" s="0">
         <v>4</v>
       </c>
       <c r="E77" t="s" s="0">
-        <v>211</v>
+        <v>225</v>
       </c>
       <c r="F77" t="s" s="0">
-        <v>212</v>
+        <v>226</v>
+      </c>
+      <c r="G77" t="s" s="0">
+        <v>4</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="s" s="0">
-        <v>204</v>
+        <v>218</v>
       </c>
       <c r="B78" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E78" t="s" s="0">
-        <v>213</v>
+        <v>227</v>
       </c>
       <c r="F78" t="s" s="0">
-        <v>214</v>
+        <v>228</v>
+      </c>
+      <c r="G78" t="s" s="0">
+        <v>46</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="s" s="0">
-        <v>215</v>
+        <v>229</v>
       </c>
       <c r="B79" t="s" s="0">
-        <v>216</v>
+        <v>230</v>
       </c>
       <c r="E79" t="s" s="0">
-        <v>217</v>
+        <v>231</v>
       </c>
       <c r="F79" t="s" s="0">
-        <v>218</v>
+        <v>232</v>
+      </c>
+      <c r="G79" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="s" s="0">
-        <v>215</v>
+        <v>229</v>
       </c>
       <c r="B80" t="s" s="0">
-        <v>219</v>
+        <v>233</v>
       </c>
       <c r="E80" t="s" s="0">
-        <v>220</v>
+        <v>234</v>
       </c>
       <c r="F80" t="s" s="0">
-        <v>221</v>
+        <v>235</v>
+      </c>
+      <c r="G80" t="s" s="0">
+        <v>236</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s" s="0">
-        <v>215</v>
+        <v>229</v>
       </c>
       <c r="B81" t="s" s="0">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="D81" t="s" s="0">
-        <v>222</v>
+        <v>237</v>
       </c>
       <c r="F81" t="s" s="0">
-        <v>223</v>
+        <v>238</v>
+      </c>
+      <c r="G81" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="s" s="0">
-        <v>215</v>
+        <v>229</v>
       </c>
       <c r="B82" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E82" t="s" s="0">
-        <v>224</v>
+        <v>239</v>
       </c>
       <c r="F82" t="s" s="0">
-        <v>225</v>
+        <v>240</v>
+      </c>
+      <c r="G82" t="s" s="0">
+        <v>46</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="s" s="0">
-        <v>215</v>
+        <v>229</v>
       </c>
       <c r="B83" t="s" s="0">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="E83" t="s" s="0">
-        <v>226</v>
+        <v>241</v>
       </c>
       <c r="F83" t="s" s="0">
-        <v>227</v>
+        <v>242</v>
+      </c>
+      <c r="G83" t="s" s="0">
+        <v>110</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="s" s="0">
-        <v>228</v>
+        <v>243</v>
       </c>
       <c r="B84" t="s" s="0">
-        <v>229</v>
+        <v>244</v>
       </c>
       <c r="E84" t="s" s="0">
-        <v>230</v>
+        <v>245</v>
       </c>
       <c r="F84" t="s" s="0">
-        <v>231</v>
+        <v>246</v>
+      </c>
+      <c r="G84" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="s" s="0">
-        <v>228</v>
+        <v>243</v>
       </c>
       <c r="B85" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E85" t="s" s="0">
-        <v>232</v>
+        <v>247</v>
       </c>
       <c r="F85" t="s" s="0">
-        <v>233</v>
+        <v>248</v>
+      </c>
+      <c r="G85" t="s" s="0">
+        <v>46</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s" s="0">
-        <v>234</v>
+        <v>249</v>
       </c>
       <c r="B86" t="s" s="0">
-        <v>235</v>
+        <v>250</v>
       </c>
       <c r="E86" t="s" s="0">
-        <v>236</v>
+        <v>251</v>
       </c>
       <c r="F86" t="s" s="0">
-        <v>237</v>
+        <v>252</v>
+      </c>
+      <c r="G86" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="s" s="0">
-        <v>234</v>
+        <v>249</v>
       </c>
       <c r="B87" t="s" s="0">
-        <v>238</v>
+        <v>253</v>
       </c>
       <c r="E87" t="s" s="0">
-        <v>239</v>
+        <v>254</v>
       </c>
       <c r="F87" t="s" s="0">
-        <v>240</v>
+        <v>255</v>
+      </c>
+      <c r="G87" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s" s="0">
-        <v>234</v>
+        <v>249</v>
       </c>
       <c r="B88" t="s" s="0">
-        <v>241</v>
+        <v>256</v>
       </c>
       <c r="E88" t="s" s="0">
-        <v>242</v>
+        <v>257</v>
       </c>
       <c r="F88" t="s" s="0">
-        <v>243</v>
+        <v>258</v>
+      </c>
+      <c r="G88" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="s" s="0">
-        <v>234</v>
+        <v>249</v>
       </c>
       <c r="B89" t="s" s="0">
-        <v>244</v>
+        <v>259</v>
       </c>
       <c r="E89" t="s" s="0">
-        <v>245</v>
+        <v>260</v>
       </c>
       <c r="F89" t="s" s="0">
-        <v>246</v>
+        <v>261</v>
+      </c>
+      <c r="G89" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s" s="0">
-        <v>234</v>
+        <v>249</v>
       </c>
       <c r="B90" t="s" s="0">
-        <v>247</v>
+        <v>262</v>
       </c>
       <c r="D90" t="s" s="0">
-        <v>248</v>
+        <v>263</v>
       </c>
       <c r="F90" t="s" s="0">
-        <v>249</v>
+        <v>264</v>
+      </c>
+      <c r="G90" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="s" s="0">
-        <v>234</v>
+        <v>249</v>
       </c>
       <c r="B91" t="s" s="0">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="D91" t="s" s="0">
-        <v>250</v>
+        <v>265</v>
       </c>
       <c r="F91" t="s" s="0">
-        <v>251</v>
+        <v>266</v>
+      </c>
+      <c r="G91" t="s" s="0">
+        <v>106</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="s" s="0">
-        <v>234</v>
+        <v>249</v>
       </c>
       <c r="B92" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E92" t="s" s="0">
-        <v>252</v>
+        <v>267</v>
       </c>
       <c r="F92" t="s" s="0">
-        <v>253</v>
+        <v>268</v>
+      </c>
+      <c r="G92" t="s" s="0">
+        <v>46</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="s" s="0">
-        <v>234</v>
+        <v>249</v>
       </c>
       <c r="B93" t="s" s="0">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="E93" t="s" s="0">
-        <v>254</v>
+        <v>269</v>
       </c>
       <c r="F93" t="s" s="0">
-        <v>255</v>
+        <v>270</v>
+      </c>
+      <c r="G93" t="s" s="0">
+        <v>110</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="s" s="0">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="B94" t="s" s="0">
-        <v>257</v>
+        <v>272</v>
       </c>
       <c r="E94" t="s" s="0">
-        <v>258</v>
+        <v>273</v>
       </c>
       <c r="F94" t="s" s="0">
-        <v>259</v>
+        <v>274</v>
+      </c>
+      <c r="G94" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="s" s="0">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="B95" t="s" s="0">
-        <v>260</v>
+        <v>275</v>
       </c>
       <c r="E95" t="s" s="0">
-        <v>261</v>
+        <v>276</v>
       </c>
       <c r="F95" t="s" s="0">
-        <v>262</v>
+        <v>277</v>
+      </c>
+      <c r="G95" t="s" s="0">
+        <v>101</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="s" s="0">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="B96" t="s" s="0">
-        <v>263</v>
+        <v>278</v>
       </c>
       <c r="E96" t="s" s="0">
-        <v>264</v>
+        <v>279</v>
       </c>
       <c r="F96" t="s" s="0">
-        <v>265</v>
+        <v>280</v>
+      </c>
+      <c r="G96" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="s" s="0">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="B97" t="s" s="0">
-        <v>266</v>
+        <v>281</v>
       </c>
       <c r="E97" t="s" s="0">
-        <v>267</v>
+        <v>282</v>
       </c>
       <c r="F97" t="s" s="0">
-        <v>268</v>
+        <v>283</v>
+      </c>
+      <c r="G97" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="s" s="0">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="B98" t="s" s="0">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="C98" t="s" s="0">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="E98" t="s" s="0">
-        <v>269</v>
+        <v>284</v>
       </c>
       <c r="F98" t="s" s="0">
-        <v>270</v>
+        <v>285</v>
+      </c>
+      <c r="G98" t="s" s="0">
+        <v>210</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="s" s="0">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="B99" t="s" s="0">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="C99" t="s" s="0">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="E99" t="s" s="0">
-        <v>269</v>
+        <v>284</v>
       </c>
       <c r="F99" t="s" s="0">
-        <v>271</v>
+        <v>286</v>
+      </c>
+      <c r="G99" t="s" s="0">
+        <v>210</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="s" s="0">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="B100" t="s" s="0">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="C100" t="s" s="0">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="E100" t="s" s="0">
-        <v>272</v>
+        <v>287</v>
       </c>
       <c r="F100" t="s" s="0">
-        <v>273</v>
+        <v>288</v>
+      </c>
+      <c r="G100" t="s" s="0">
+        <v>210</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="s" s="0">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="B101" t="s" s="0">
-        <v>274</v>
+        <v>289</v>
       </c>
       <c r="E101" t="s" s="0">
-        <v>275</v>
+        <v>290</v>
       </c>
       <c r="F101" t="s" s="0">
-        <v>276</v>
+        <v>291</v>
+      </c>
+      <c r="G101" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="s" s="0">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="B102" t="s" s="0">
-        <v>277</v>
+        <v>292</v>
       </c>
       <c r="E102" t="s" s="0">
-        <v>278</v>
+        <v>293</v>
       </c>
       <c r="F102" t="s" s="0">
-        <v>279</v>
+        <v>294</v>
+      </c>
+      <c r="G102" t="s" s="0">
+        <v>236</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="s" s="0">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="B103" t="s" s="0">
-        <v>280</v>
+        <v>295</v>
       </c>
       <c r="E103" t="s" s="0">
-        <v>281</v>
+        <v>296</v>
       </c>
       <c r="F103" t="s" s="0">
-        <v>282</v>
+        <v>297</v>
+      </c>
+      <c r="G103" t="s" s="0">
+        <v>101</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="s" s="0">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="B104" t="s" s="0">
-        <v>283</v>
+        <v>298</v>
       </c>
       <c r="E104" t="s" s="0">
-        <v>284</v>
+        <v>299</v>
       </c>
       <c r="F104" t="s" s="0">
-        <v>285</v>
+        <v>300</v>
+      </c>
+      <c r="G104" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="s" s="0">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="B105" t="s" s="0">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="D105" t="s" s="0">
-        <v>286</v>
+        <v>301</v>
       </c>
       <c r="F105" t="s" s="0">
-        <v>287</v>
+        <v>302</v>
+      </c>
+      <c r="G105" t="s" s="0">
+        <v>106</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="s" s="0">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="B106" t="s" s="0">
-        <v>201</v>
+        <v>215</v>
       </c>
       <c r="E106" t="s" s="0">
-        <v>288</v>
+        <v>303</v>
       </c>
       <c r="F106" t="s" s="0">
-        <v>289</v>
+        <v>304</v>
+      </c>
+      <c r="G106" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="s" s="0">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="B107" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E107" t="s" s="0">
-        <v>290</v>
+        <v>305</v>
       </c>
       <c r="F107" t="s" s="0">
-        <v>291</v>
+        <v>306</v>
+      </c>
+      <c r="G107" t="s" s="0">
+        <v>46</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="s" s="0">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="B108" t="s" s="0">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="E108" t="s" s="0">
-        <v>292</v>
+        <v>307</v>
       </c>
       <c r="F108" t="s" s="0">
-        <v>293</v>
+        <v>308</v>
+      </c>
+      <c r="G108" t="s" s="0">
+        <v>110</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="s" s="0">
-        <v>294</v>
+        <v>309</v>
       </c>
       <c r="B109" t="s" s="0">
-        <v>295</v>
+        <v>310</v>
       </c>
       <c r="E109" t="s" s="0">
-        <v>296</v>
+        <v>311</v>
       </c>
       <c r="F109" t="s" s="0">
-        <v>297</v>
+        <v>312</v>
+      </c>
+      <c r="G109" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="s" s="0">
-        <v>294</v>
+        <v>309</v>
       </c>
       <c r="B110" t="s" s="0">
-        <v>298</v>
+        <v>313</v>
       </c>
       <c r="D110" t="s" s="0">
-        <v>299</v>
+        <v>314</v>
       </c>
       <c r="F110" t="s" s="0">
-        <v>300</v>
+        <v>315</v>
+      </c>
+      <c r="G110" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="s" s="0">
-        <v>294</v>
+        <v>309</v>
       </c>
       <c r="B111" t="s" s="0">
-        <v>208</v>
+        <v>222</v>
       </c>
       <c r="E111" t="s" s="0">
-        <v>301</v>
+        <v>316</v>
       </c>
       <c r="F111" t="s" s="0">
-        <v>302</v>
+        <v>317</v>
+      </c>
+      <c r="G111" t="s" s="0">
+        <v>50</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="s" s="0">
-        <v>294</v>
+        <v>309</v>
       </c>
       <c r="B112" t="s" s="0">
         <v>4</v>
       </c>
       <c r="E112" t="s" s="0">
-        <v>303</v>
+        <v>318</v>
       </c>
       <c r="F112" t="s" s="0">
-        <v>304</v>
+        <v>319</v>
+      </c>
+      <c r="G112" t="s" s="0">
+        <v>4</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="s" s="0">
-        <v>294</v>
+        <v>309</v>
       </c>
       <c r="B113" t="s" s="0">
-        <v>305</v>
+        <v>320</v>
       </c>
       <c r="E113" t="s" s="0">
-        <v>306</v>
+        <v>321</v>
       </c>
       <c r="F113" t="s" s="0">
-        <v>307</v>
+        <v>322</v>
+      </c>
+      <c r="G113" t="s" s="0">
+        <v>323</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="s" s="0">
-        <v>294</v>
+        <v>309</v>
       </c>
       <c r="B114" t="s" s="0">
-        <v>308</v>
+        <v>324</v>
       </c>
       <c r="E114" t="s" s="0">
-        <v>309</v>
+        <v>325</v>
       </c>
       <c r="F114" t="s" s="0">
-        <v>310</v>
+        <v>326</v>
+      </c>
+      <c r="G114" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="s" s="0">
-        <v>294</v>
+        <v>309</v>
       </c>
       <c r="B115" t="s" s="0">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="D115" t="s" s="0">
-        <v>311</v>
+        <v>327</v>
       </c>
       <c r="F115" t="s" s="0">
-        <v>312</v>
+        <v>328</v>
+      </c>
+      <c r="G115" t="s" s="0">
+        <v>106</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="s" s="0">
-        <v>294</v>
+        <v>309</v>
       </c>
       <c r="B116" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E116" t="s" s="0">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="F116" t="s" s="0">
-        <v>314</v>
+        <v>330</v>
+      </c>
+      <c r="G116" t="s" s="0">
+        <v>46</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="s" s="0">
-        <v>294</v>
+        <v>309</v>
       </c>
       <c r="B117" t="s" s="0">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="E117" t="s" s="0">
-        <v>315</v>
+        <v>331</v>
       </c>
       <c r="F117" t="s" s="0">
-        <v>316</v>
+        <v>332</v>
+      </c>
+      <c r="G117" t="s" s="0">
+        <v>110</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="s" s="0">
-        <v>317</v>
+        <v>333</v>
       </c>
       <c r="B118" t="s" s="0">
-        <v>318</v>
+        <v>334</v>
       </c>
       <c r="E118" t="s" s="0">
-        <v>319</v>
+        <v>335</v>
       </c>
       <c r="F118" t="s" s="0">
-        <v>320</v>
+        <v>336</v>
+      </c>
+      <c r="G118" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="s" s="0">
-        <v>317</v>
+        <v>333</v>
       </c>
       <c r="B119" t="s" s="0">
-        <v>321</v>
+        <v>337</v>
       </c>
       <c r="E119" t="s" s="0">
-        <v>322</v>
+        <v>338</v>
       </c>
       <c r="F119" t="s" s="0">
-        <v>323</v>
+        <v>339</v>
+      </c>
+      <c r="G119" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="s" s="0">
-        <v>317</v>
+        <v>333</v>
       </c>
       <c r="B120" t="s" s="0">
-        <v>324</v>
+        <v>340</v>
       </c>
       <c r="E120" t="s" s="0">
-        <v>325</v>
+        <v>341</v>
       </c>
       <c r="F120" t="s" s="0">
-        <v>326</v>
+        <v>342</v>
+      </c>
+      <c r="G120" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="s" s="0">
-        <v>317</v>
+        <v>333</v>
       </c>
       <c r="B121" t="s" s="0">
-        <v>327</v>
+        <v>343</v>
       </c>
       <c r="E121" t="s" s="0">
-        <v>328</v>
+        <v>344</v>
       </c>
       <c r="F121" t="s" s="0">
-        <v>329</v>
+        <v>345</v>
+      </c>
+      <c r="G121" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="s" s="0">
-        <v>317</v>
+        <v>333</v>
       </c>
       <c r="B122" t="s" s="0">
-        <v>164</v>
+        <v>177</v>
       </c>
       <c r="D122" t="s" s="0">
-        <v>330</v>
+        <v>346</v>
       </c>
       <c r="F122" t="s" s="0">
-        <v>331</v>
+        <v>347</v>
+      </c>
+      <c r="G122" t="s" s="0">
+        <v>29</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="s" s="0">
-        <v>317</v>
+        <v>333</v>
       </c>
       <c r="B123" t="s" s="0">
-        <v>305</v>
+        <v>320</v>
       </c>
       <c r="E123" t="s" s="0">
-        <v>332</v>
+        <v>348</v>
       </c>
       <c r="F123" t="s" s="0">
-        <v>333</v>
+        <v>349</v>
+      </c>
+      <c r="G123" t="s" s="0">
+        <v>323</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="s" s="0">
-        <v>317</v>
+        <v>333</v>
       </c>
       <c r="B124" t="s" s="0">
-        <v>334</v>
+        <v>350</v>
       </c>
       <c r="E124" t="s" s="0">
-        <v>335</v>
+        <v>351</v>
       </c>
       <c r="F124" t="s" s="0">
-        <v>336</v>
+        <v>352</v>
+      </c>
+      <c r="G124" t="s" s="0">
+        <v>33</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="s" s="0">
-        <v>317</v>
+        <v>333</v>
       </c>
       <c r="B125" t="s" s="0">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="D125" t="s" s="0">
-        <v>337</v>
+        <v>353</v>
       </c>
       <c r="F125" t="s" s="0">
-        <v>338</v>
+        <v>354</v>
+      </c>
+      <c r="G125" t="s" s="0">
+        <v>106</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="s" s="0">
-        <v>317</v>
+        <v>333</v>
       </c>
       <c r="B126" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E126" t="s" s="0">
-        <v>339</v>
+        <v>355</v>
       </c>
       <c r="F126" t="s" s="0">
-        <v>340</v>
+        <v>356</v>
+      </c>
+      <c r="G126" t="s" s="0">
+        <v>46</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="s" s="0">
-        <v>317</v>
+        <v>333</v>
       </c>
       <c r="B127" t="s" s="0">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="E127" t="s" s="0">
-        <v>341</v>
+        <v>357</v>
       </c>
       <c r="F127" t="s" s="0">
-        <v>342</v>
+        <v>358</v>
+      </c>
+      <c r="G127" t="s" s="0">
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>